<commit_message>
rag + open inference + arizePhoenix integration success
</commit_message>
<xml_diff>
--- a/rag_demo/reference/note.xlsx
+++ b/rag_demo/reference/note.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ai_action\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{655CC020-11E5-483A-9E34-5F0FDBE4D549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC6DE7A-B1E3-4C2C-8799-F5D550B33AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summay" sheetId="1" r:id="rId1"/>
-    <sheet name="notes" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="RAG" sheetId="2" r:id="rId2"/>
+    <sheet name="arize_phoenix" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,13 +34,115 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="4">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="4">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>生成SRS,登录github,vpn ok</t>
   </si>
   <si>
-    <t>1.生成ssh key, add to github</t>
+    <t>申请了deepseek apikey 作为chatmodel, 千问 apikey 做为embedding model</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用docker 启动了 pgvector</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#4. 查询 vector table created
+PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker exec rag-postgres psql -U postgres -d rag_db -c "\dt"
+              List of relations
+ Schema |       Name       | Type  |  Owner   
+--------+------------------+-------+----------
+ public | knowledge_vector | table | postgres
+(1 row)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://localhost:8080/api/test/chat</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://localhost:8080/api/test/chat/stream</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>测试使用deepseek api call 成功 （stream 和 non-stream）</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1. 启动postgresql db 
+PS D:\workspace\github\rag\rag_demo\src\main\docker&gt;docker compose up -d</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#2. 查看 pgvectoer 容器名字
+PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker ps 
+CONTAINER ID   IMAGE                                              COMMAND                   CREATED          STATUS                    PORTS                                         NAMES
+14c511256a4d   pgvector/pgvector:0.8.6-pg16                       "docker-entrypoint.s…"   19 minutes ago   Up 19 minutes (healthy)   0.0.0.0:5432-&gt;5432/tcp, [::]:5432-&gt;5432/tcp   rag-postgres</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#3.验证 pgvector 扩展是否生效
+PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker exec rag-postgres psql -U postgres -d rag_db -c "\dx"
+                             List of installed extensions
+  Name   | Version |   Schema   |                     Description
+---------+---------+------------+------------------------------------------------------
+ plpgsql | 1.0     | pg_catalog | PL/pgSQL procedural language
+ vector  | 0.8.6   | public     | vector data type and ivfflat and hnsw access methods
+(2 rows)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>PS C:\Users\杨圣&gt; ssh-keygen -t ed25519 -C "526884815@qq.com"
@@ -66,70 +168,129 @@
 |               . |
 +----[SHA256]-----+
 PS C:\Users\杨圣&gt;</t>
-  </si>
-  <si>
-    <t>申请了deepseek apikey 作为chatmodel, 千问 apikey 做为embedding model</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用docker 启动了 pgvector</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>#4. 查询 vector table created
-PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker exec rag-postgres psql -U postgres -d rag_db -c "\dt"
-              List of relations
- Schema |       Name       | Type  |  Owner   
---------+------------------+-------+----------
- public | knowledge_vector | table | postgres
-(1 row)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://localhost:8080/api/test/chat</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>测试 deepseek API call success (non-stream)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>测试 deepseek api call (stream)</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://localhost:8080/api/test/chat/stream</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>测试使用deepseek api call 成功 （stream 和 non-stream）</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用docker 启动 pgvector 容器(postgresql db + 安装vector 扩展)， 用作rag 的embedding 数据库</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>#1. 启动postgresql db 
-PS D:\workspace\github\rag\rag_demo\src\main\docker&gt;docker compose up -d</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>#2. 查看 pgvectoer 容器名字
-PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker ps 
-CONTAINER ID   IMAGE                                              COMMAND                   CREATED          STATUS                    PORTS                                         NAMES
-14c511256a4d   pgvector/pgvector:0.8.6-pg16                       "docker-entrypoint.s…"   19 minutes ago   Up 19 minutes (healthy)   0.0.0.0:5432-&gt;5432/tcp, [::]:5432-&gt;5432/tcp   rag-postgres</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>#3.验证 pgvector 扩展是否生效
-PS D:\workspace\github\rag\rag_demo\src\main\docker&gt; docker exec rag-postgres psql -U postgres -d rag_db -c "\dx"
-                             List of installed extensions
-  Name   | Version |   Schema   |                     Description
----------+---------+------------+------------------------------------------------------
- plpgsql | 1.0     | pg_catalog | PL/pgSQL procedural language
- vector  | 0.8.6   | public     | vector data type and ivfflat and hnsw access methods
-(2 rows)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1.生成ssh key, add to github</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.使用docker 启动 pgvector 容器(postgresql db + 安装vector 扩展)， 用作rag 的embedding 数据库</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#5测试 deepseek API call success (non-stream)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#6.测试 deepseek api call (stream)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#7. 测试 千问embedding bean created
+GET:http://localhost:8080/api/test/embedding/health</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#8. 验证 通义千问 text-embedding-v3 生效，应该是1024维度
+POST: http://localhost:8080/api/test/embedding/test</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">验证 通义千问 text-embedding-v3 生效 </t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>测试Rag</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1.删旧表，让 LangChain4j 用默认结构重建（4 列：embedding_id/embedding/text/metadata）
+docker exec rag-postgres psql -U postgres -d rag_db -c "DROP TABLE IF EXISTS knowledge_vector;"
+docker exec rag-postgres psql -U postgres -d rag_db -c "DROP TABLE IF EXISTS knowledge_vector;"
+DROP TABLE</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#2. 测试ingest 一句话</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>#3 rag 测试成功。
+## 1. 入库（如果之前的数据还在就不用重复跑）
+Invoke-RestMethod -Uri http://localhost:8080/api/rag/ingest -Method POST -ContentType "application/json" -Body '{
+  "content": "RAG (Retrieval-Augmented Generation) is a technique that combines information retrieval with text generation. pgvector is a PostgreSQL extension that supports vector similarity search with HNSW and IVFFlat indexes. HNSW is the recommended index type for most RAG scenarios because it offers fast queries and high recall.",
+  "source": "rag-intro.md"
+}'
+## 2. RAG 问答（DeepSeek 基于你入库的内容回答）
+Invoke-RestMethod -Uri http://localhost:8080/api/rag/chat -Method POST -ContentType "application/json" -Body '{"question":"What index types does pgvector support and which is best for RAG?"}'
+预期 DeepSeek 回答里会提到 HNSW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>​</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 和 IVFFlat，并且说 HNSW 更适合 RAG —— 这就证明它不是在瞎编，是真的从你入库的文档里检索到了信息再生成的。
+</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>rag embedding 到pgvector成功</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>rag 测试成功，deepseek 作为chat Model, qwen-text-embedding-v3 embedding model, pgVector向量数据库</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1. 启动 Phoenix（Docker）
+用 Docker 一条命令启动 Phoenix（含 UI + OTLP collector）：
+docker run -d --name phoenix `
+  -p 6006:6006 `
+  -p 4317:4317 `
+  -e PHOENIX_PORT=6006 `
+  arizephoenix/phoenix:latest</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#2. 验证
+docker ps | findstr phoenix
+PS D:\workspace\github\rag\rag_demo&gt;  docker ps | findStr phoenix
+b41504bdc20c   arizephoenix/phoenix:latest                        "/usr/bin/python3.13??   3 minutes ago   Up 3 minutes              0.0.0.0:4317-&gt;4317/tcp, [::]:4317-&gt;4317/tcp, 0.0.0.0:6006-&gt;6006/tcp, [::]:6006-&gt;6006/tcp   phoenix</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#3. 浏览器打开 http://localhost:6006
+​ —— 应该能看到 Phoenix 的空仪表盘。</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>embedding 成功， deepseek chat 成功</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>optl + open inference 成功， Arize Phoenix 集成成功</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#4. ArizePhoenix 集成成功</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -137,7 +298,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,6 +335,13 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -183,12 +351,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -200,15 +383,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
@@ -216,14 +396,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -247,15 +442,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>63501</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>9436695</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>36</xdr:row>
       <xdr:rowOff>34089</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -291,15 +486,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>44450</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>9414641</xdr:colOff>
-      <xdr:row>74</xdr:row>
+      <xdr:row>71</xdr:row>
       <xdr:rowOff>140045</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -333,7 +528,262 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7226671</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>139890</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="图片 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B970EA7F-5953-1484-4025-1DADB875D5D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3143250" y="21513800"/>
+          <a:ext cx="7226671" cy="3695890"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7741048</xdr:colOff>
+      <xdr:row>130</xdr:row>
+      <xdr:rowOff>101879</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="图片 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8107DE2-10F5-2BB2-430D-3D45F8FF4E09}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3143250" y="25958800"/>
+          <a:ext cx="7741048" cy="5435879"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>137</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>10268473</xdr:colOff>
+      <xdr:row>164</xdr:row>
+      <xdr:rowOff>127251</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="图片 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28116DE4-F089-253F-8B06-E78331675D6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="32581850"/>
+          <a:ext cx="10173223" cy="4883401"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>654050</xdr:colOff>
+      <xdr:row>168</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>10986031</xdr:colOff>
+      <xdr:row>199</xdr:row>
+      <xdr:rowOff>25682</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="图片 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFC50CED-F5DE-7156-9F6B-DF6C59831B9A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3797300" y="42779950"/>
+          <a:ext cx="10331981" cy="5493032"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -586,15 +1036,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:B5"/>
+  <dimension ref="A2:B10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.54296875" customWidth="1"/>
-    <col min="2" max="2" width="41.54296875" customWidth="1"/>
+    <col min="2" max="2" width="102" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>46235</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -602,27 +1052,67 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>46257</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>3</v>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>46257</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>4</v>
+      <c r="B4" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>46257</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>10</v>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>46258</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46259</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -634,83 +1124,686 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:C43"/>
+  <dimension ref="A2:B168"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.6328125" customWidth="1"/>
-    <col min="2" max="2" width="0.90625" customWidth="1"/>
-    <col min="3" max="3" width="190.7265625" customWidth="1"/>
+    <col min="1" max="1" width="45" customWidth="1"/>
+    <col min="2" max="2" width="190.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="2:3" ht="254.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    <row r="2" spans="1:2" ht="322" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" ht="28" x14ac:dyDescent="0.25">
-      <c r="C8" s="5" t="s">
+      <c r="B2" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+    </row>
+    <row r="5" spans="1:2" ht="28" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="2:3" ht="70" x14ac:dyDescent="0.25">
-      <c r="C9" s="5" t="s">
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="70" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="112" x14ac:dyDescent="0.25">
+      <c r="A7" s="10"/>
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="98" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="6"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="112" x14ac:dyDescent="0.25">
-      <c r="C10" s="5" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="6"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
+      <c r="B18" s="6"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="6"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="10"/>
+      <c r="B22" s="6"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="6"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="6"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="6"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="6"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="6"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="6"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="6"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="10"/>
+      <c r="B30" s="6"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="10"/>
+      <c r="B31" s="6"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="6"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="6"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="10"/>
+      <c r="B34" s="6"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="6"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="10"/>
+      <c r="B36" s="6"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="10"/>
+      <c r="B37" s="6"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="10"/>
+      <c r="B38" s="6"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="10"/>
+      <c r="B39" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="112" x14ac:dyDescent="0.25">
-      <c r="C11" s="5" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="10"/>
+      <c r="B40" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14">
-        <v>3</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C15" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B42">
-        <v>4</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="7" t="s">
-        <v>9</v>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="10"/>
+      <c r="B41" s="6"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="10"/>
+      <c r="B42" s="6"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="10"/>
+      <c r="B43" s="6"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="10"/>
+      <c r="B44" s="6"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="10"/>
+      <c r="B45" s="6"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="10"/>
+      <c r="B46" s="6"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="10"/>
+      <c r="B47" s="6"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="10"/>
+      <c r="B48" s="6"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="10"/>
+      <c r="B49" s="6"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="10"/>
+      <c r="B50" s="6"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="10"/>
+      <c r="B51" s="6"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="10"/>
+      <c r="B52" s="6"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="10"/>
+      <c r="B53" s="6"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="10"/>
+      <c r="B54" s="6"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="10"/>
+      <c r="B55" s="6"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="10"/>
+      <c r="B56" s="6"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="10"/>
+      <c r="B57" s="6"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="10"/>
+      <c r="B58" s="6"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="10"/>
+      <c r="B59" s="6"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="10"/>
+      <c r="B60" s="6"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="10"/>
+      <c r="B61" s="6"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="10"/>
+      <c r="B62" s="6"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="10"/>
+      <c r="B63" s="6"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="10"/>
+      <c r="B64" s="6"/>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="10"/>
+      <c r="B65" s="6"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="10"/>
+      <c r="B66" s="6"/>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="10"/>
+      <c r="B67" s="6"/>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="10"/>
+      <c r="B68" s="6"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="10"/>
+      <c r="B69" s="6"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="10"/>
+      <c r="B70" s="6"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="10"/>
+      <c r="B71" s="6"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="10"/>
+      <c r="B72" s="6"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="10"/>
+      <c r="B73" s="6"/>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="10"/>
+      <c r="B74" s="6"/>
+    </row>
+    <row r="75" spans="1:2" ht="28" x14ac:dyDescent="0.25">
+      <c r="A75" s="10"/>
+      <c r="B75" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="10"/>
+      <c r="B76" s="6"/>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="10"/>
+      <c r="B77" s="6"/>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="10"/>
+      <c r="B78" s="6"/>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="10"/>
+      <c r="B79" s="6"/>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="10"/>
+      <c r="B80" s="6"/>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="10"/>
+      <c r="B81" s="6"/>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="10"/>
+      <c r="B82" s="6"/>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="10"/>
+      <c r="B83" s="6"/>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="10"/>
+      <c r="B84" s="6"/>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="10"/>
+      <c r="B85" s="6"/>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="10"/>
+      <c r="B86" s="6"/>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="10"/>
+      <c r="B87" s="6"/>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="10"/>
+      <c r="B88" s="6"/>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="10"/>
+      <c r="B89" s="6"/>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="10"/>
+      <c r="B90" s="6"/>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="10"/>
+      <c r="B91" s="6"/>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="10"/>
+      <c r="B92" s="6"/>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="10"/>
+      <c r="B93" s="6"/>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="10"/>
+      <c r="B94" s="6"/>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="10"/>
+      <c r="B95" s="6"/>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" s="10"/>
+      <c r="B96" s="6"/>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" s="10"/>
+      <c r="B97" s="6"/>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" s="10"/>
+      <c r="B98" s="6"/>
+    </row>
+    <row r="99" spans="1:2" ht="28" x14ac:dyDescent="0.25">
+      <c r="A99" s="10"/>
+      <c r="B99" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" s="10"/>
+      <c r="B100" s="6"/>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" s="10"/>
+      <c r="B101" s="6"/>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" s="10"/>
+      <c r="B102" s="6"/>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" s="10"/>
+      <c r="B103" s="6"/>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" s="10"/>
+      <c r="B104" s="6"/>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" s="10"/>
+      <c r="B105" s="6"/>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" s="10"/>
+      <c r="B106" s="6"/>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="10"/>
+      <c r="B107" s="6"/>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" s="10"/>
+      <c r="B108" s="6"/>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="10"/>
+      <c r="B109" s="6"/>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" s="10"/>
+      <c r="B110" s="6"/>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" s="10"/>
+      <c r="B111" s="6"/>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" s="10"/>
+      <c r="B112" s="6"/>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" s="10"/>
+      <c r="B113" s="6"/>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" s="10"/>
+      <c r="B114" s="6"/>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" s="10"/>
+      <c r="B115" s="6"/>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" s="10"/>
+      <c r="B116" s="6"/>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" s="10"/>
+      <c r="B117" s="6"/>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" s="10"/>
+      <c r="B118" s="6"/>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" s="10"/>
+      <c r="B119" s="6"/>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" s="10"/>
+      <c r="B120" s="6"/>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" s="10"/>
+      <c r="B121" s="6"/>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" s="10"/>
+      <c r="B122" s="6"/>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" s="10"/>
+      <c r="B123" s="6"/>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" s="10"/>
+      <c r="B124" s="6"/>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" s="10"/>
+      <c r="B125" s="6"/>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" s="10"/>
+      <c r="B126" s="6"/>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" s="10"/>
+      <c r="B127" s="6"/>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" s="10"/>
+      <c r="B128" s="6"/>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" s="10"/>
+      <c r="B129" s="6"/>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" s="10"/>
+      <c r="B130" s="6"/>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" s="10"/>
+      <c r="B131" s="6"/>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132" s="10"/>
+      <c r="B132" s="6"/>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133" s="10"/>
+      <c r="B133" s="6"/>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134" s="10"/>
+      <c r="B134" s="6"/>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135" s="6"/>
+      <c r="B135" s="6"/>
+    </row>
+    <row r="136" spans="1:2" ht="70" x14ac:dyDescent="0.25">
+      <c r="A136" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137" s="6"/>
+      <c r="B137" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138" s="6"/>
+      <c r="B138" s="6"/>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139" s="6"/>
+      <c r="B139" s="6"/>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140" s="6"/>
+      <c r="B140" s="6"/>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141" s="6"/>
+      <c r="B141" s="6"/>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142" s="6"/>
+      <c r="B142" s="6"/>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143" s="6"/>
+      <c r="B143" s="6"/>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" s="6"/>
+      <c r="B144" s="6"/>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" s="6"/>
+      <c r="B145" s="6"/>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146" s="6"/>
+      <c r="B146" s="6"/>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147" s="6"/>
+      <c r="B147" s="6"/>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" s="6"/>
+      <c r="B148" s="6"/>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" s="6"/>
+      <c r="B149" s="6"/>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" s="6"/>
+      <c r="B150" s="6"/>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" s="6"/>
+      <c r="B151" s="6"/>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" s="6"/>
+      <c r="B152" s="6"/>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" s="6"/>
+      <c r="B153" s="6"/>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" s="6"/>
+      <c r="B154" s="6"/>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" s="6"/>
+      <c r="B155" s="6"/>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" s="6"/>
+      <c r="B156" s="6"/>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" s="6"/>
+      <c r="B157" s="6"/>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" s="6"/>
+      <c r="B158" s="6"/>
+    </row>
+    <row r="168" spans="2:2" ht="182" x14ac:dyDescent="0.25">
+      <c r="B168" s="11" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:A134"/>
+  </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C15" r:id="rId1" xr:uid="{97143255-371E-4F54-9F6B-B685976E193C}"/>
-    <hyperlink ref="C43" r:id="rId2" xr:uid="{317AF21E-8084-4F1B-9F85-419C2D8FA991}"/>
+    <hyperlink ref="B12" r:id="rId1" xr:uid="{97143255-371E-4F54-9F6B-B685976E193C}"/>
+    <hyperlink ref="B40" r:id="rId2" xr:uid="{317AF21E-8084-4F1B-9F85-419C2D8FA991}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -720,9 +1813,53 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="B3:B13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="169" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:2" ht="112" x14ac:dyDescent="0.25">
+      <c r="B3" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" ht="112" x14ac:dyDescent="0.25">
+      <c r="B4" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" ht="394" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" ht="383" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
add how to start in local, and enable pg db connection via Intellij
</commit_message>
<xml_diff>
--- a/rag_demo/reference/note.xlsx
+++ b/rag_demo/reference/note.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ai_action\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC6DE7A-B1E3-4C2C-8799-F5D550B33AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20CD1783-9525-4051-B624-77E57338A61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summay" sheetId="1" r:id="rId1"/>
-    <sheet name="RAG" sheetId="2" r:id="rId2"/>
+    <sheet name="rag" sheetId="2" r:id="rId2"/>
     <sheet name="arize_phoenix" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="4">
+  <futureMetadata name="XLRICHVALUE" count="5">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -68,8 +68,15 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="4">
+  <valueMetadata count="5">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -82,12 +89,15 @@
     <bk>
       <rc t="1" v="3"/>
     </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>生成SRS,登录github,vpn ok</t>
   </si>
@@ -291,6 +301,10 @@
   </si>
   <si>
     <t>#4. ArizePhoenix 集成成功</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>#5， 查看 postgresql db data , from database tool in intellij</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -748,7 +762,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
   <rv s="0">
     <v>0</v>
     <v>5</v>
@@ -763,6 +777,10 @@
   </rv>
   <rv s="0">
     <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -783,6 +801,7 @@
   <rel r:id="rId2"/>
   <rel r:id="rId3"/>
   <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
 </richValueRels>
 </file>
 
@@ -1813,7 +1832,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B3:B13"/>
+  <dimension ref="B3:B18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="169" customWidth="1"/>
@@ -1859,6 +1878,17 @@
         <v>#VALUE!</v>
       </c>
     </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" ht="119.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>